<commit_message>
Dev interfunc 22022024: - grote aanpassing: isgfunc.c + isgfunc.h - kleine aanpassing (naamgeving gewijzigd) isgfunc_prio.c - reg.c diverse plaatsen wat commentaar toegevoegd - paar kleine aanpassingen reg.c met name naamgeving aangeroepte functies + commentaar
</commit_message>
<xml_diff>
--- a/ISG bespreekpunten sessie Ton.xlsx
+++ b/ISG bespreekpunten sessie Ton.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26924"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27126"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ccapp\source\repos\CodingConnected\TLCGenExampleController\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1ACDE63F-90D1-40C5-ACB3-A51113F7B707}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1182F1B-967E-4E32-8840-2D8A4EBD637A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{98A45D7C-0F26-427C-8C08-BF5B78174C08}"/>
+    <workbookView xWindow="1470" yWindow="1470" windowWidth="21600" windowHeight="11295" activeTab="1" xr2:uid="{98A45D7C-0F26-427C-8C08-BF5B78174C08}"/>
   </bookViews>
   <sheets>
-    <sheet name="Blad1" sheetId="1" r:id="rId1"/>
+    <sheet name="Bespreekpunten" sheetId="1" r:id="rId1"/>
+    <sheet name="TODO lijst" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,10 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
-  <si>
-    <t>ISG uitzoekpunten</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
   <si>
     <t>Stel bij de Kruispunt 123456 2 en 62 zijn groen er is geen aanvraag voor 9 en 26 heeftt de AAPR opstaan. 28 mag nu alternatief realisieren. 9 vraag opeens wel aan. Nu kan de maximale wachttijd van 26 hoger worden. Dus of 9 had niet meer mogen komen of 28 had niet alternatief mogen realiseren omdat de beurt van 9 nog open stond. Zou Ton dit niet kunnen oplossen?</t>
   </si>
@@ -49,6 +47,63 @@
   <si>
     <t xml:space="preserve">Nu we in TLCGen een wachtijdvoorspeller hebben, kunnen we ook een flowdiagram laten meelopen met de voorspelling van de eerst volgende cyclus. Het is alleen voor de de show dus het mag niet te veel kosten. Wat denk jij?
 </t>
+  </si>
+  <si>
+    <t>maximale wachttijd loopt niet continue af maar hikt af en toe. Dat komt omdat het blok pas op einde CV van alle richtingen wordt doorgegeven (en tot dat moment nog steeds een richting primair (maximaal) mag realiseren)?</t>
+  </si>
+  <si>
+    <t>Is door de extra loopjes de funcites</t>
+  </si>
+  <si>
+    <t>Hoe om te gaan als een voetgangers net voor einde groen nog bij wil komen (maximale wachttijd altijd hiervoor reserveren)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Huidige implementatie is dat fietsers / voetgangers (hard) meeverlengen met parallelle auto en meerealiseren. Sommige wegbeheerders willen voetgangers / fietsers niet laten meekomen. Hoe daar mee om te gaan </t>
+  </si>
+  <si>
+    <t>Hoe om te gaan met va- ontruimen (voor UC3 als fileingreep maar wat kiezen we bij WTV-ers)</t>
+  </si>
+  <si>
+    <t>Hoe om te gaan met file stroomop- afwaarts (en verkorten / verlengen groentijden)</t>
+  </si>
+  <si>
+    <t>Hoe om te gaan met PTP ingrepen  ?</t>
+  </si>
+  <si>
+    <t>ISG bespreekpunten</t>
+  </si>
+  <si>
+    <t>To do ISG:</t>
+  </si>
+  <si>
+    <t>PG_OVERSLAG wordt soms niet snel genoeg gezet i.c.m. alternatieve realisaties.. Ton’s hulp hierin zou ik zeer op prijs stellen.</t>
+  </si>
+  <si>
+    <t>Wachttijdvoorspeller voor meerdere realisaties. Ook hier zou ik Ton’s hulp goed kunnen gebruiken.</t>
+  </si>
+  <si>
+    <t>Robuuste groentijdverdeler.</t>
+  </si>
+  <si>
+    <t>Niet tegelijk realisren deel conflicten. Bijv. PG_overslag zetten bij geen aanvraag of blokkeren en geen conflicterend groen.</t>
+  </si>
+  <si>
+    <t>3 delige oversteken is een special.</t>
+  </si>
+  <si>
+    <t>Gelijktijdig realiserende voedende richtingen waarvan de volgrichting conlficterend zijn is ook een special.</t>
+  </si>
+  <si>
+    <t>VA-ontruimen.</t>
+  </si>
+  <si>
+    <t>Halfstar.</t>
+  </si>
+  <si>
+    <t>TVG wordt nu alleen lager bij een file-ingreep. Niet blokkeren.</t>
+  </si>
+  <si>
+    <t>De laatste 3 items zouden we tijdelijk kunnen disableen,   </t>
   </si>
 </sst>
 </file>
@@ -98,10 +153,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standaard" xfId="0" builtinId="0"/>
@@ -416,12 +472,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DDB3D780-F54C-4102-8725-157B1F55941B}">
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
@@ -429,7 +485,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -437,7 +493,7 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -446,6 +502,127 @@
       </c>
       <c r="B4" t="s">
         <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11" t="s">
+        <v>2</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BBACE92F-5579-4428-AAAF-90597438A88D}">
+  <dimension ref="A1:A14"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>